<commit_message>
Initial Senior Citizen Care project
</commit_message>
<xml_diff>
--- a/sample_data.xlsx
+++ b/sample_data.xlsx
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E33"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -465,130 +465,521 @@
         <v>senior.test@seniorcare.local</v>
       </c>
       <c r="B4" t="str">
-        <v>Lakshmi Devi</v>
+        <v>Kalyani Ammal</v>
       </c>
       <c r="C4" t="str">
         <v>senior_citizen</v>
       </c>
       <c r="D4" t="str">
-        <v>+91 98765 43210</v>
+        <v>+91 9080578504</v>
       </c>
       <c r="E4" t="str">
-        <v>Flat 104, Senior Haven, Adyar, Chennai</v>
+        <v>Door No. 14, 2nd Cross Street, Kasturibai Nagar, Adyar, Chennai</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>family.test@seniorcare.local</v>
+        <v>senior2.test@seniorcare.local</v>
       </c>
       <c r="B5" t="str">
-        <v>Priya Ramesh</v>
+        <v>Ramasamy Sundaram</v>
       </c>
       <c r="C5" t="str">
-        <v>family_member</v>
+        <v>senior_citizen</v>
       </c>
       <c r="D5" t="str">
-        <v>+91 98765 00003</v>
+        <v>+91 98765 43211</v>
       </c>
       <c r="E5" t="str">
-        <v>Velachery, Chennai</v>
+        <v>Flat 2A, Anandam Apts, 4th Main Road, Gandhi Nagar, Adyar, Chennai</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>family2.test@seniorcare.local</v>
+        <v>senior3.test@seniorcare.local</v>
       </c>
       <c r="B6" t="str">
-        <v>Vignesh Ramesh</v>
+        <v>Meenakshi Ammal</v>
       </c>
       <c r="C6" t="str">
-        <v>family_member</v>
+        <v>senior_citizen</v>
       </c>
       <c r="D6" t="str">
-        <v>+91 98765 00006</v>
+        <v>+91 98765 43212</v>
       </c>
       <c r="E6" t="str">
-        <v>Adyar, Chennai</v>
+        <v>Old No. 45, New No. 22, South Mada Street, Mylapore, Chennai</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>caretaker.test@seniorcare.local</v>
+        <v>senior4.test@seniorcare.local</v>
       </c>
       <c r="B7" t="str">
-        <v>Anitha Krishnan</v>
+        <v>Gopalakrishnan V</v>
       </c>
       <c r="C7" t="str">
-        <v>caretaker</v>
+        <v>senior_citizen</v>
       </c>
       <c r="D7" t="str">
-        <v>+91 98765 00004</v>
+        <v>+91 98765 43213</v>
       </c>
       <c r="E7" t="str">
-        <v>Mylapore, Chennai</v>
+        <v>Plot 88, 3rd Seaward Road, Valmiki Nagar, Thiruvanmiyur, Chennai</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>caregiver.test@seniorcare.local</v>
+        <v>senior5.test@seniorcare.local</v>
       </c>
       <c r="B8" t="str">
-        <v>Anitha Krishnan</v>
+        <v>Dr. K. S. Ramanathan</v>
       </c>
       <c r="C8" t="str">
-        <v>caretaker</v>
+        <v>senior_citizen</v>
       </c>
       <c r="D8" t="str">
-        <v>+91 98765 00004</v>
+        <v>+91 98765 43215</v>
       </c>
       <c r="E8" t="str">
-        <v>Mylapore, Chennai</v>
+        <v>Door No. 28, 4th Seaward Road, Valmiki Nagar, Thiruvanmiyur, Chennai</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>volunteer.test@seniorcare.local</v>
+        <v>senior6.test@seniorcare.local</v>
       </c>
       <c r="B9" t="str">
-        <v>Karthik Raman</v>
+        <v>Rajalakshmi Narayanan</v>
       </c>
       <c r="C9" t="str">
-        <v>volunteer</v>
+        <v>senior_citizen</v>
       </c>
       <c r="D9" t="str">
-        <v>+91 98765 00005</v>
+        <v>+91 98765 43216</v>
       </c>
       <c r="E9" t="str">
-        <v>Thiruvanmiyur, Chennai</v>
+        <v>Flat 3B, Brindavan Apts, 3rd Cross Street, Mandaveli, Chennai</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>temp.caregiver@seniorcare.local</v>
+        <v>family.test@seniorcare.local</v>
       </c>
       <c r="B10" t="str">
-        <v>Dinesh Kumar (Probation)</v>
+        <v>Bhavana Lakshmi (Daughter)</v>
       </c>
       <c r="C10" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D10" t="str">
+        <v>+91 9345403336</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Velachery, Chennai</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>bhavanalakshmi12006@gmail.com</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Bhavana Lakshmi (Daughter)</v>
+      </c>
+      <c r="C11" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D11" t="str">
+        <v>+91 9345403336</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Velachery, Chennai</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>arun.kumar@seniorcare.local</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Arun Kumar (Son)</v>
+      </c>
+      <c r="C12" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D12" t="str">
+        <v>+91 98765 77771</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Velachery, Chennai</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>pooja.lakshmi@seniorcare.local</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Pooja Lakshmi (Daughter)</v>
+      </c>
+      <c r="C13" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D13" t="str">
+        <v>+91 98765 77772</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Velachery, Chennai</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>family2.test@seniorcare.local</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Suresh Sundaram (Son)</v>
+      </c>
+      <c r="C14" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D14" t="str">
+        <v>+91 98765 11111</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Adyar, Chennai</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>suresh.sundaram@seniorcare.local</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Suresh Sundaram (Son)</v>
+      </c>
+      <c r="C15" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D15" t="str">
+        <v>+91 98765 11111</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Adyar, Chennai</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>kavitha.sundaram@seniorcare.local</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Kavitha Sundaram (Daughter)</v>
+      </c>
+      <c r="C16" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D16" t="str">
+        <v>+91 98765 11112</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Adyar, Chennai</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>family3.test@seniorcare.local</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Geetha Mohan (Daughter-in-law)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D17" t="str">
+        <v>+91 98765 22222</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Mylapore, Chennai</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>geetha.mohan@seniorcare.local</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Geetha Mohan (Daughter-in-law)</v>
+      </c>
+      <c r="C18" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D18" t="str">
+        <v>+91 98765 22222</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Mylapore, Chennai</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>mohan.narayanan@seniorcare.local</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Mohan Narayanan (Son)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D19" t="str">
+        <v>+91 98765 22223</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Mylapore, Chennai</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>family4.test@seniorcare.local</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Venkat Gopal (Son-in-law)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D20" t="str">
+        <v>+91 98765 33333</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Thiruvanmiyur, Chennai</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>venkat.gopal@seniorcare.local</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Venkat Gopal (Son-in-law)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D21" t="str">
+        <v>+91 98765 33333</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Thiruvanmiyur, Chennai</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>shanthi.gopal@seniorcare.local</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Shanthi Gopal (Daughter)</v>
+      </c>
+      <c r="C22" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D22" t="str">
+        <v>+91 98765 33334</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Thiruvanmiyur, Chennai</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>family5.test@seniorcare.local</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Dr. Karthik Ramanathan (Son)</v>
+      </c>
+      <c r="C23" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D23" t="str">
+        <v>+91 98765 55551</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Thiruvanmiyur, Chennai</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>karthik.ramanathan@seniorcare.local</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Dr. Karthik Ramanathan (Son)</v>
+      </c>
+      <c r="C24" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D24" t="str">
+        <v>+91 98765 55551</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Thiruvanmiyur, Chennai</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>priya.ramanathan@seniorcare.local</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Priya Ramanathan (Daughter)</v>
+      </c>
+      <c r="C25" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D25" t="str">
+        <v>+91 98765 55552</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Besant Nagar, Chennai</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>ashwin.ramanathan@seniorcare.local</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Ashwin Ramanathan (Son)</v>
+      </c>
+      <c r="C26" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D26" t="str">
+        <v>+91 98765 55553</v>
+      </c>
+      <c r="E26" t="str">
+        <v>OMR, Chennai</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>family6.test@seniorcare.local</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Deepa Narayanan (Daughter)</v>
+      </c>
+      <c r="C27" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D27" t="str">
+        <v>+91 98765 66661</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Mandaveli, Chennai</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>deepa.narayanan@seniorcare.local</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Deepa Narayanan (Daughter)</v>
+      </c>
+      <c r="C28" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D28" t="str">
+        <v>+91 98765 66661</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Mandaveli, Chennai</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>vijay.narayanan@seniorcare.local</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Vijay Narayanan (Son)</v>
+      </c>
+      <c r="C29" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D29" t="str">
+        <v>+91 98765 66662</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Alwarpet, Chennai</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>swetha.narayanan@seniorcare.local</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Swetha Narayanan (Daughter)</v>
+      </c>
+      <c r="C30" t="str">
+        <v>family_member</v>
+      </c>
+      <c r="D30" t="str">
+        <v>+91 98765 66663</v>
+      </c>
+      <c r="E30" t="str">
+        <v>RA Puram, Chennai</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>caretaker.test@seniorcare.local</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Anitha Krishnan</v>
+      </c>
+      <c r="C31" t="str">
         <v>caretaker</v>
       </c>
-      <c r="D10" t="str">
-        <v>+91 98765 00099</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Tambaram, Chennai</v>
+      <c r="D31" t="str">
+        <v>+91 6382598599</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Mylapore, Chennai</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>caregiver.test@seniorcare.local</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Anitha Krishnan</v>
+      </c>
+      <c r="C32" t="str">
+        <v>caretaker</v>
+      </c>
+      <c r="D32" t="str">
+        <v>+91 6382598599</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Mylapore, Chennai</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>volunteer.test@seniorcare.local</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Karthik Raman</v>
+      </c>
+      <c r="C33" t="str">
+        <v>volunteer</v>
+      </c>
+      <c r="D33" t="str">
+        <v>+91 9443327744</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Thiruvanmiyur, Chennai</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E33"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -621,10 +1012,10 @@
         <v>FEE-301</v>
       </c>
       <c r="B2" t="str">
-        <v>Lakshmi Devi</v>
+        <v>Kalyani Ammal</v>
       </c>
       <c r="C2" t="str">
-        <v>October 2026 Monthly Care &amp; Assisted Living</v>
+        <v>October 2026 Monthly Care &amp; Assisted Living Package</v>
       </c>
       <c r="D2" t="str">
         <v>Monthly Care</v>
@@ -633,33 +1024,33 @@
         <v>12000</v>
       </c>
       <c r="F2">
-        <v>8000</v>
+        <v>12000</v>
       </c>
       <c r="G2">
-        <v>4000</v>
+        <v>0</v>
       </c>
       <c r="H2" t="str">
-        <v>Partially Paid</v>
+        <v>Paid</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>FEE-302</v>
+        <v>FEE-304</v>
       </c>
       <c r="B3" t="str">
-        <v>Ramasamy Sundaram</v>
+        <v>Kalyani Ammal</v>
       </c>
       <c r="C3" t="str">
-        <v>Physiotherapy Package (10 Sessions)</v>
+        <v>Dr. S. Kumar Geriatric Consultation &amp; 12-Lead ECG</v>
       </c>
       <c r="D3" t="str">
-        <v>Physiotherapy</v>
+        <v>Doctor Consultation</v>
       </c>
       <c r="E3">
-        <v>5000</v>
+        <v>1500</v>
       </c>
       <c r="F3">
-        <v>5000</v>
+        <v>1500</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -670,48 +1061,48 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>FEE-303</v>
+        <v>FEE-305</v>
       </c>
       <c r="B4" t="str">
-        <v>Meenakshi Ammal</v>
+        <v>Kalyani Ammal</v>
       </c>
       <c r="C4" t="str">
-        <v>Specialist Geriatric Consultation &amp; Labs</v>
+        <v>Apollo Pharmacy Monthly Tablets Refill (BP &amp; Sugar)</v>
       </c>
       <c r="D4" t="str">
-        <v>Medical Consultation</v>
+        <v>Pharmacy &amp; Medicine</v>
       </c>
       <c r="E4">
-        <v>3500</v>
+        <v>2450</v>
       </c>
       <c r="F4">
+        <v>2450</v>
+      </c>
+      <c r="G4">
         <v>0</v>
       </c>
-      <c r="G4">
-        <v>3500</v>
-      </c>
       <c r="H4" t="str">
-        <v>Overdue</v>
+        <v>Paid</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>FEE-304</v>
+        <v>FEE-306</v>
       </c>
       <c r="B5" t="str">
-        <v>Lakshmi Devi</v>
+        <v>Kalyani Ammal</v>
       </c>
       <c r="C5" t="str">
-        <v>Dietary Nutrition Plan (Quarterly)</v>
+        <v>Diagnostics: Complete Blood Count &amp; Fasting Lipid Profile</v>
       </c>
       <c r="D5" t="str">
-        <v>Meals</v>
+        <v>Lab Diagnostics</v>
       </c>
       <c r="E5">
-        <v>4500</v>
+        <v>1800</v>
       </c>
       <c r="F5">
-        <v>4500</v>
+        <v>1800</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -720,9 +1111,61 @@
         <v>Paid</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>FEE-307</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Kalyani Ammal</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Physiotherapy &amp; Mobility Rehabilitation (5 Sessions)</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Physiotherapy</v>
+      </c>
+      <c r="E6">
+        <v>3000</v>
+      </c>
+      <c r="F6">
+        <v>3000</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Paid</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>FEE-302</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Ramasamy Sundaram</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Post-op Knee Rehabilitation (10 Sessions)</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Physiotherapy</v>
+      </c>
+      <c r="E7">
+        <v>5000</v>
+      </c>
+      <c r="F7">
+        <v>5000</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Paid</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -820,7 +1263,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -853,7 +1296,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Lakshmi Devi</v>
+        <v>Kalyani Ammal</v>
       </c>
       <c r="B2">
         <v>72</v>
@@ -862,22 +1305,22 @@
         <v>Female</v>
       </c>
       <c r="D2" t="str">
-        <v>+91 98765 43210</v>
+        <v>+91 9080578504</v>
       </c>
       <c r="E2" t="str">
-        <v>Room 104</v>
+        <v>Independent Home Residence</v>
       </c>
       <c r="F2" t="str">
         <v>O+</v>
       </c>
       <c r="G2" t="str">
-        <v>Hypertension, Mild Type-2 Diabetes. Regular morning BP check needed.</v>
+        <v>Hypertension, Mild Type-2 Diabetes. Monthly routine checkup cycle scheduled.</v>
       </c>
       <c r="H2" t="str">
-        <v>Priya Ramesh (Daughter)</v>
+        <v>Bhavana Lakshmi (Daughter)</v>
       </c>
       <c r="I2" t="str">
-        <v>+91 98765 00003</v>
+        <v>+91 9345403336</v>
       </c>
     </row>
     <row r="3">
@@ -894,7 +1337,7 @@
         <v>+91 98765 43211</v>
       </c>
       <c r="E3" t="str">
-        <v>Room 108</v>
+        <v>Independent Residence</v>
       </c>
       <c r="F3" t="str">
         <v>B+</v>
@@ -923,7 +1366,7 @@
         <v>+91 98765 43212</v>
       </c>
       <c r="E4" t="str">
-        <v>Room 202</v>
+        <v>Independent Residence</v>
       </c>
       <c r="F4" t="str">
         <v>A+</v>
@@ -932,7 +1375,7 @@
         <v>Mild memory lapses, arthritis, cataract surgery scheduled.</v>
       </c>
       <c r="H4" t="str">
-        <v>Geetha Mohan (Niece)</v>
+        <v>Geetha Mohan (Daughter-in-law)</v>
       </c>
       <c r="I4" t="str">
         <v>+91 98765 22222</v>
@@ -952,7 +1395,7 @@
         <v>+91 98765 43213</v>
       </c>
       <c r="E5" t="str">
-        <v>Room 205</v>
+        <v>Independent Residence</v>
       </c>
       <c r="F5" t="str">
         <v>AB+</v>
@@ -961,7 +1404,7 @@
         <v>Pacemaker implanted 2022, routine cardiac review.</v>
       </c>
       <c r="H5" t="str">
-        <v>Venkat G (Son)</v>
+        <v>Venkat Gopal (Son-in-law)</v>
       </c>
       <c r="I5" t="str">
         <v>+91 98765 33333</v>
@@ -969,43 +1412,101 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Dr. K. S. Ramanathan</v>
+      </c>
+      <c r="B6">
+        <v>76</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D6" t="str">
+        <v>+91 98765 43215</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Villa 12, Senior Care Haven</v>
+      </c>
+      <c r="F6" t="str">
+        <v>A+</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Chronic hypertension, diabetic neuropathy, needs monthly cardiology review.</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Dr. Karthik Ramanathan (Son)</v>
+      </c>
+      <c r="I6" t="str">
+        <v>+91 98765 55551</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Rajalakshmi Narayanan</v>
+      </c>
+      <c r="B7">
+        <v>74</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Female</v>
+      </c>
+      <c r="D7" t="str">
+        <v>+91 98765 43216</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Suite 104, Senior Care Haven</v>
+      </c>
+      <c r="F7" t="str">
+        <v>B+</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Osteoarthritis, mild glaucoma, routine eye drops &amp; physiotherapy.</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Deepa Narayanan (Daughter)</v>
+      </c>
+      <c r="I7" t="str">
+        <v>+91 98765 66661</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
         <v>Saraswathi Natarajan</v>
       </c>
-      <c r="B6">
+      <c r="B8">
         <v>69</v>
       </c>
-      <c r="C6" t="str">
+      <c r="C8" t="str">
         <v>Female</v>
       </c>
-      <c r="D6" t="str">
+      <c r="D8" t="str">
         <v>+91 98765 43214</v>
       </c>
-      <c r="E6" t="str">
-        <v>Room 301</v>
-      </c>
-      <c r="F6" t="str">
+      <c r="E8" t="str">
+        <v>Independent Residence</v>
+      </c>
+      <c r="F8" t="str">
         <v>O-</v>
       </c>
-      <c r="G6" t="str">
+      <c r="G8" t="str">
         <v>Asthma, inhaler on bedside table.</v>
       </c>
-      <c r="H6" t="str">
+      <c r="H8" t="str">
         <v>Natarajan S (Husband)</v>
       </c>
-      <c r="I6" t="str">
+      <c r="I8" t="str">
         <v>+91 98765 44444</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1026,24 +1527,313 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Priya Ramesh</v>
+        <v>Bhavana Lakshmi (Daughter)</v>
       </c>
       <c r="B2" t="str">
-        <v>+91 98765 00003</v>
+        <v>+91 9345403336</v>
       </c>
       <c r="C2" t="str">
-        <v>family.test@seniorcare.local</v>
+        <v>bhavanalakshmi12006@gmail.com</v>
       </c>
       <c r="D2" t="str">
         <v>Daughter</v>
       </c>
       <c r="E2" t="str">
-        <v>Lakshmi Devi</v>
+        <v>Kalyani Ammal</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Bhavana Lakshmi (Daughter)</v>
+      </c>
+      <c r="B3" t="str">
+        <v>+91 9345403336</v>
+      </c>
+      <c r="C3" t="str">
+        <v>family.test@seniorcare.local</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Daughter</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Kalyani Ammal</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Arun Kumar (Son)</v>
+      </c>
+      <c r="B4" t="str">
+        <v>+91 98765 77771</v>
+      </c>
+      <c r="C4" t="str">
+        <v>arun.kumar@seniorcare.local</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Son</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Kalyani Ammal</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Pooja Lakshmi (Daughter)</v>
+      </c>
+      <c r="B5" t="str">
+        <v>+91 98765 77772</v>
+      </c>
+      <c r="C5" t="str">
+        <v>pooja.lakshmi@seniorcare.local</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Daughter</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Kalyani Ammal</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Suresh Sundaram (Son)</v>
+      </c>
+      <c r="B6" t="str">
+        <v>+91 98765 11111</v>
+      </c>
+      <c r="C6" t="str">
+        <v>family2.test@seniorcare.local</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Son</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Ramasamy Sundaram</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Kavitha Sundaram (Daughter)</v>
+      </c>
+      <c r="B7" t="str">
+        <v>+91 98765 11112</v>
+      </c>
+      <c r="C7" t="str">
+        <v>kavitha.sundaram@seniorcare.local</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Daughter</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Ramasamy Sundaram</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Geetha Mohan (Daughter-in-law)</v>
+      </c>
+      <c r="B8" t="str">
+        <v>+91 98765 22222</v>
+      </c>
+      <c r="C8" t="str">
+        <v>family3.test@seniorcare.local</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Daughter-in-law</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Meenakshi Ammal</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Mohan Narayanan (Son)</v>
+      </c>
+      <c r="B9" t="str">
+        <v>+91 98765 22223</v>
+      </c>
+      <c r="C9" t="str">
+        <v>mohan.narayanan@seniorcare.local</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Son</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Meenakshi Ammal</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Venkat Gopal (Son-in-law)</v>
+      </c>
+      <c r="B10" t="str">
+        <v>+91 98765 33333</v>
+      </c>
+      <c r="C10" t="str">
+        <v>family4.test@seniorcare.local</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Son-in-law</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Gopalakrishnan V</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Shanthi Gopal (Daughter)</v>
+      </c>
+      <c r="B11" t="str">
+        <v>+91 98765 33334</v>
+      </c>
+      <c r="C11" t="str">
+        <v>shanthi.gopal@seniorcare.local</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Daughter</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Gopalakrishnan V</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Dr. Karthik Ramanathan (Son)</v>
+      </c>
+      <c r="B12" t="str">
+        <v>+91 98765 55551</v>
+      </c>
+      <c r="C12" t="str">
+        <v>family5.test@seniorcare.local</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Son</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Dr. K. S. Ramanathan</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Dr. Karthik Ramanathan (Son)</v>
+      </c>
+      <c r="B13" t="str">
+        <v>+91 98765 55551</v>
+      </c>
+      <c r="C13" t="str">
+        <v>karthik.ramanathan@seniorcare.local</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Son</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Dr. K. S. Ramanathan</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Priya Ramanathan (Daughter)</v>
+      </c>
+      <c r="B14" t="str">
+        <v>+91 98765 55552</v>
+      </c>
+      <c r="C14" t="str">
+        <v>priya.ramanathan@seniorcare.local</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Daughter</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Dr. K. S. Ramanathan</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Ashwin Ramanathan (Son)</v>
+      </c>
+      <c r="B15" t="str">
+        <v>+91 98765 55553</v>
+      </c>
+      <c r="C15" t="str">
+        <v>ashwin.ramanathan@seniorcare.local</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Son</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Dr. K. S. Ramanathan</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Deepa Narayanan (Daughter)</v>
+      </c>
+      <c r="B16" t="str">
+        <v>+91 98765 66661</v>
+      </c>
+      <c r="C16" t="str">
+        <v>family6.test@seniorcare.local</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Daughter</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Rajalakshmi Narayanan</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Deepa Narayanan (Daughter)</v>
+      </c>
+      <c r="B17" t="str">
+        <v>+91 98765 66661</v>
+      </c>
+      <c r="C17" t="str">
+        <v>deepa.narayanan@seniorcare.local</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Daughter</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Rajalakshmi Narayanan</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Vijay Narayanan (Son)</v>
+      </c>
+      <c r="B18" t="str">
+        <v>+91 98765 66662</v>
+      </c>
+      <c r="C18" t="str">
+        <v>vijay.narayanan@seniorcare.local</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Son</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Rajalakshmi Narayanan</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Swetha Narayanan (Daughter)</v>
+      </c>
+      <c r="B19" t="str">
+        <v>+91 98765 66663</v>
+      </c>
+      <c r="C19" t="str">
+        <v>swetha.narayanan@seniorcare.local</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Daughter</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Rajalakshmi Narayanan</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1152,7 +1942,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1173,7 +1963,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Lakshmi Devi</v>
+        <v>Kalyani Ammal</v>
       </c>
       <c r="B2" t="str">
         <v>safe</v>
@@ -1185,12 +1975,12 @@
         <v>Feeling great today, completed morning walk.</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-10-05T15:17:46.973Z</v>
+        <v>2026-10-08T10:47:10.579Z</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Lakshmi Devi</v>
+        <v>Kalyani Ammal</v>
       </c>
       <c r="B3" t="str">
         <v>safe</v>
@@ -1202,12 +1992,12 @@
         <v>Took morning medications on time.</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-10-04T15:17:46.973Z</v>
+        <v>2026-10-07T10:47:10.579Z</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Lakshmi Devi</v>
+        <v>Kalyani Ammal</v>
       </c>
       <c r="B4" t="str">
         <v>safe</v>
@@ -1219,7 +2009,7 @@
         <v>Slight joint ache, applied ointment.</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-10-03T15:17:46.973Z</v>
+        <v>2026-10-06T10:47:10.579Z</v>
       </c>
     </row>
     <row r="5">
@@ -1236,7 +2026,7 @@
         <v>Physiotherapy exercises done.</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-10-05T15:17:46.973Z</v>
+        <v>2026-10-08T10:47:10.579Z</v>
       </c>
     </row>
     <row r="6">
@@ -1253,7 +2043,7 @@
         <v>All good, had breakfast.</v>
       </c>
       <c r="E6" t="str">
-        <v>2026-10-05T15:17:46.973Z</v>
+        <v>2026-10-08T10:47:10.579Z</v>
       </c>
     </row>
     <row r="7">
@@ -1270,12 +2060,46 @@
         <v>Resting comfortably.</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-10-04T15:17:46.973Z</v>
+        <v>2026-10-07T10:47:10.579Z</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Dr. K. S. Ramanathan</v>
+      </c>
+      <c r="B8" t="str">
+        <v>safe</v>
+      </c>
+      <c r="C8" t="str">
+        <v>good</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Morning vitals stable, blood pressure 125/82 mmHg.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2026-10-08T10:47:10.579Z</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Rajalakshmi Narayanan</v>
+      </c>
+      <c r="B9" t="str">
+        <v>safe</v>
+      </c>
+      <c r="C9" t="str">
+        <v>good</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Eye drops taken and morning prayers done.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2026-10-08T10:47:10.579Z</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1309,7 +2133,7 @@
         <v>EMG-1024</v>
       </c>
       <c r="B2" t="str">
-        <v>Lakshmi Devi</v>
+        <v>Kalyani Ammal</v>
       </c>
       <c r="C2" t="str">
         <v>active</v>
@@ -1318,10 +2142,10 @@
         <v>critical</v>
       </c>
       <c r="E2" t="str">
-        <v>Room 104 - Bedside</v>
+        <v>Home Residence - Bedside (Adyar)</v>
       </c>
       <c r="F2" t="str">
-        <v>Severe shortness of breath reported. Caregiver dispatched.</v>
+        <v>Severe shortness of breath reported. Caregiver dispatched to home.</v>
       </c>
     </row>
     <row r="3">
@@ -1353,7 +2177,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1383,19 +2207,19 @@
         <v>APT-201</v>
       </c>
       <c r="B2" t="str">
-        <v>Lakshmi Devi</v>
+        <v>Kalyani Ammal</v>
       </c>
       <c r="C2" t="str">
-        <v>Dr. S. Kumar, MD (Cardiology)</v>
+        <v>Dr. S. Kumar, MD (Geriatric Cardiology)</v>
       </c>
       <c r="D2" t="str">
-        <v>Cardiology</v>
+        <v>Geriatric Medicine</v>
       </c>
       <c r="E2" t="str">
         <v>Apollo Senior Health Center</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-10-06 10:30 AM</v>
+        <v>2026-10-09 10:00 AM</v>
       </c>
       <c r="G2" t="str">
         <v>Upcoming</v>
@@ -1403,45 +2227,45 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>APT-202</v>
+        <v>APT-195</v>
       </c>
       <c r="B3" t="str">
-        <v>Ramasamy Sundaram</v>
+        <v>Kalyani Ammal</v>
       </c>
       <c r="C3" t="str">
-        <v>Dr. R. Malathi, MS (Ophthalmology)</v>
+        <v>Dr. S. Kumar, MD (Geriatric Cardiology)</v>
       </c>
       <c r="D3" t="str">
-        <v>Ophthalmology</v>
+        <v>Geriatric Medicine</v>
       </c>
       <c r="E3" t="str">
-        <v>Sankara Nethralaya</v>
+        <v>Apollo Senior Health Center</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-10-08 02:00 PM</v>
+        <v>2026-10-06 09:30 AM</v>
       </c>
       <c r="G3" t="str">
-        <v>Upcoming</v>
+        <v>Completed</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>APT-203</v>
+        <v>APT-202</v>
       </c>
       <c r="B4" t="str">
-        <v>Meenakshi Ammal</v>
+        <v>Ramasamy Sundaram</v>
       </c>
       <c r="C4" t="str">
-        <v>Dr. P. Vijay, MS (Orthopedics)</v>
+        <v>Dr. R. Malathi, MS (Ophthalmology)</v>
       </c>
       <c r="D4" t="str">
-        <v>Orthopedics</v>
+        <v>Ophthalmology</v>
       </c>
       <c r="E4" t="str">
-        <v>Fortis Malar Hospital</v>
+        <v>Sankara Nethralaya</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-10-10 11:15 AM</v>
+        <v>2026-10-11 02:00 PM</v>
       </c>
       <c r="G4" t="str">
         <v>Upcoming</v>
@@ -1449,37 +2273,83 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>APT-195</v>
+        <v>APT-203</v>
       </c>
       <c r="B5" t="str">
-        <v>Lakshmi Devi</v>
+        <v>Meenakshi Ammal</v>
       </c>
       <c r="C5" t="str">
-        <v>Dr. K. Narayanan (General Physician)</v>
+        <v>Dr. P. Vijay, MS (Orthopedics)</v>
       </c>
       <c r="D5" t="str">
-        <v>General Medicine</v>
+        <v>Orthopedics</v>
       </c>
       <c r="E5" t="str">
+        <v>Fortis Malar Hospital</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-10-13 11:15 AM</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Upcoming</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>APT-204</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Dr. K. S. Ramanathan</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Dr. S. Kumar, MD (Geriatric Cardiology)</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Cardiology</v>
+      </c>
+      <c r="E6" t="str">
         <v>Apollo Senior Health Center</v>
       </c>
-      <c r="F5" t="str">
-        <v>2026-09-28 09:30 AM</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Completed</v>
+      <c r="F6" t="str">
+        <v>2026-10-10 10:30 AM</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Upcoming</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>APT-205</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Rajalakshmi Narayanan</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Dr. R. Malathi, MS (Ophthalmology)</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Ophthalmology</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Sankara Nethralaya</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-10-12 03:30 PM</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Upcoming</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1503,7 +2373,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Lakshmi Devi</v>
+        <v>Kalyani Ammal</v>
       </c>
       <c r="B2" t="str">
         <v>Medicine Pickup</v>
@@ -1523,7 +2393,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Lakshmi Devi</v>
+        <v>Kalyani Ammal</v>
       </c>
       <c r="B3" t="str">
         <v>Food Assistance</v>
@@ -1581,9 +2451,49 @@
         <v>Unassigned</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Dr. K. S. Ramanathan</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Medicine Pickup</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Monthly Cardiac Medications Refill &amp; Glucometer Strips</v>
+      </c>
+      <c r="D6" t="str">
+        <v>High</v>
+      </c>
+      <c r="E6" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Karthik Raman (Volunteer)</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Rajalakshmi Narayanan</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Food Assistance</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Low-Salt Herbal Soup &amp; Diabetic Dinner Delivery</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Normal</v>
+      </c>
+      <c r="E7" t="str">
+        <v>In Progress</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Anitha Krishnan (Caregiver)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>